<commit_message>
Tennis PostPlanner export update 2026-06-25
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRKECGsgNjjnTtQV4Sg3fC
</commit_message>
<xml_diff>
--- a/Tennis/postplanner-imports/tfr-postplanner-2026-06-25.xlsx
+++ b/Tennis/postplanner-imports/tfr-postplanner-2026-06-25.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/25/2026  12:48</t>
+          <t>06/25/2026  13:02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06/25/2026  14:18</t>
+          <t>06/25/2026  14:31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -505,7 +505,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06/25/2026  15:48</t>
+          <t>06/25/2026  16:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -519,7 +519,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06/25/2026  17:18</t>
+          <t>06/25/2026  17:29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -533,7 +533,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/25/2026  18:48</t>
+          <t>06/25/2026  18:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -546,7 +546,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/25/2026  20:18</t>
+          <t>06/25/2026  20:27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>